<commit_message>
feat: implement script to generate differentiated educational reading and math assessment documents in docx format
</commit_message>
<xml_diff>
--- a/Homework/Homework_Levels.xlsx
+++ b/Homework/Homework_Levels.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dsuth\Documents\Joshua\Homework\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C7904B72-DD6C-4572-BF05-C0B8AE909414}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93BB7023-B2ED-49C6-BF50-641B822DF851}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4680" yWindow="4680" windowWidth="28800" windowHeight="15345" xr2:uid="{1687B906-C1FF-4971-BCD9-598C6DE83F52}"/>
+    <workbookView xWindow="5070" yWindow="5070" windowWidth="28800" windowHeight="15345" xr2:uid="{1687B906-C1FF-4971-BCD9-598C6DE83F52}"/>
   </bookViews>
   <sheets>
     <sheet name="Homework_Levels" sheetId="1" r:id="rId1"/>
@@ -517,7 +517,7 @@
         <v>2</v>
       </c>
       <c r="B4">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -525,7 +525,7 @@
         <v>3</v>
       </c>
       <c r="B5">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -645,7 +645,7 @@
         <v>18</v>
       </c>
       <c r="B20">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add Week 3 homework documents and update assessment levels file
</commit_message>
<xml_diff>
--- a/Homework/Homework_Levels.xlsx
+++ b/Homework/Homework_Levels.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dsuth\Documents\Joshua\Homework\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93BB7023-B2ED-49C6-BF50-641B822DF851}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E26F222F-1501-4B83-9767-368E4CD94E9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5070" yWindow="5070" windowWidth="28800" windowHeight="15345" xr2:uid="{1687B906-C1FF-4971-BCD9-598C6DE83F52}"/>
+    <workbookView xWindow="4395" yWindow="4605" windowWidth="20460" windowHeight="10770" xr2:uid="{1687B906-C1FF-4971-BCD9-598C6DE83F52}"/>
   </bookViews>
   <sheets>
     <sheet name="Homework_Levels" sheetId="1" r:id="rId1"/>
@@ -481,6 +481,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB78EC63-B8E4-421B-A7B3-2935F7D84FB5}">
   <dimension ref="A1:D20"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="27" customWidth="1"/>
+    <col min="2" max="2" width="39" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
@@ -581,7 +585,7 @@
         <v>10</v>
       </c>
       <c r="B12">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">

</xml_diff>